<commit_message>
ClaudeFinanceLab reviews 1g, 2 and 3: exit-multiple basis, selected comps range
DCF review (DCF Model Builder):
- Report the implied exit multiple on a FY2029 year-end basis (10.3x); keep 9.9x mid-year
- New WACC x exit-multiple grid (sens_wacc_exit_multiple.csv); price implies 35x FY2029 EBITDA
- Raw-beta cross-check ($351); terminal FCF uplift explained; stub shown both ways
- Excel: year-end multiple, market EV / FY2029 EBITDA, new reconciliation check (ALL OK)

Comps review (Comparable Company Analysis):
- Walmart-alone column; selected range anchored on Tier 1 with Walmart ceiling (~$450-$690)
- EV/Revenue and P/S shown but not used; dollar stores as reference only
- Albertsons/Sprouts/PriceSmart rationale, EBITDAR and DLTR limitations, sum-of-the-parts test

Forecast follow-up: FCF definition (SBC add-back) and interest assumptions added to packet 03.
Memo, deck, football field and README updated. 101 tests pass.
</commit_message>
<xml_diff>
--- a/outputs/COST_Valuation_Model.xlsx
+++ b/outputs/COST_Valuation_Model.xlsx
@@ -5424,7 +5424,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="492">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="495">
   <si>
     <t xml:space="preserve">Costco Wholesale Corporation (COST): Equity Research and Valuation Model</t>
   </si>
@@ -6578,7 +6578,10 @@
     <t xml:space="preserve">Share price 31 Jan 2025 ($)</t>
   </si>
   <si>
-    <t xml:space="preserve">Implied terminal EV / FY2029 EBITDA</t>
+    <t xml:space="preserve">Implied terminal EV / FY2029 EBITDA (mid-year basis)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implied terminal EV / FY2029 EBITDA (FY2029 year-end basis; compare with trading multiples)</t>
   </si>
   <si>
     <t xml:space="preserve">Net cash</t>
@@ -6587,6 +6590,9 @@
     <t xml:space="preserve">Market EV (market cap - net cash)</t>
   </si>
   <si>
+    <t xml:space="preserve">Market EV / FY2029E EBITDA</t>
+  </si>
+  <si>
     <t xml:space="preserve">Market EV / FY2025E EBITDA</t>
   </si>
   <si>
@@ -6885,6 +6891,9 @@
   </si>
   <si>
     <t xml:space="preserve">FY2025 EPS ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implied exit multiple, FY2029 year-end basis</t>
   </si>
   <si>
     <t xml:space="preserve">Sensitivity grid centre = base value ($)</t>
@@ -7739,7 +7748,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="7" t="str">
-        <f aca="false">Checks!E22</f>
+        <f aca="false">Checks!E23</f>
         <v>ALL OK</v>
       </c>
     </row>
@@ -7897,7 +7906,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7907,26 +7916,26 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B6" s="68" t="n">
         <f aca="false">Sensitivity!B40</f>
@@ -7943,7 +7952,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B7" s="56" t="n">
         <f aca="false">MIN(Sensitivity!C11:E13)</f>
@@ -7960,7 +7969,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B8" s="68" t="n">
         <f aca="false">Comps!C37</f>
@@ -7977,7 +7986,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B9" s="68" t="n">
         <f aca="false">Comps!C39</f>
@@ -7994,7 +8003,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B10" s="68" t="n">
         <f aca="false">Comps!C38</f>
@@ -8011,7 +8020,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B11" s="68" t="n">
         <f aca="false">Comps!F37</f>
@@ -8024,7 +8033,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="C13" s="69" t="n">
         <f aca="false">DCF!B49</f>
@@ -8033,7 +8042,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C14" s="70" t="n">
         <f aca="false">Sensitivity!B42</f>
@@ -8042,7 +8051,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="C15" s="71" t="n">
         <f aca="false">DCF!B50</f>
@@ -8065,7 +8074,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
@@ -8087,29 +8096,29 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B6" s="72" t="n">
         <f aca="false">SUMPRODUCT(ABS(Forecast!C54:H54))</f>
@@ -8129,7 +8138,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B7" s="72" t="n">
         <f aca="false">SUMPRODUCT(ABS(Forecast!D33:H33-Forecast!C33:G33-Forecast!D67:H67))</f>
@@ -8149,7 +8158,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B8" s="74" t="n">
         <f aca="false">Forecast!C18</f>
@@ -8169,7 +8178,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B9" s="74" t="n">
         <f aca="false">Forecast!H18</f>
@@ -8189,7 +8198,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B10" s="74" t="n">
         <f aca="false">Forecast!H21</f>
@@ -8209,7 +8218,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B11" s="74" t="n">
         <f aca="false">Forecast!D28</f>
@@ -8329,58 +8338,58 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B17" s="74" t="n">
-        <f aca="false">Sensitivity!D12</f>
-        <v>336.683667848478</v>
+        <f aca="false">DCF!B52</f>
+        <v>10.3234520203114</v>
       </c>
       <c r="C17" s="73" t="n">
-        <v>336.683667848477</v>
+        <v>10.3234520203114</v>
       </c>
       <c r="D17" s="72" t="n">
         <f aca="false">B17-C17</f>
         <v>0</v>
       </c>
       <c r="E17" s="12" t="str">
-        <f aca="false">IF(ABS(D17)&lt;=0.05,"OK","CHECK")</f>
+        <f aca="false">IF(ABS(D17)&lt;=0.005,"OK","CHECK")</f>
         <v>OK</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B18" s="74" t="n">
+        <f aca="false">Sensitivity!D12</f>
+        <v>336.683667848478</v>
+      </c>
+      <c r="C18" s="73" t="n">
+        <v>336.683667848477</v>
+      </c>
+      <c r="D18" s="72" t="n">
+        <f aca="false">B18-C18</f>
+        <v>0</v>
+      </c>
+      <c r="E18" s="12" t="str">
+        <f aca="false">IF(ABS(D18)&lt;=0.05,"OK","CHECK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>491</v>
+      </c>
+      <c r="B19" s="74" t="n">
         <f aca="false">Comps!G31</f>
         <v>36.5402556760886</v>
       </c>
-      <c r="C18" s="73" t="n">
+      <c r="C19" s="73" t="n">
         <v>36.5402</v>
-      </c>
-      <c r="D18" s="72" t="n">
-        <f aca="false">B18-C18</f>
-        <v>5.5676088621226E-005</v>
-      </c>
-      <c r="E18" s="12" t="str">
-        <f aca="false">IF(ABS(D18)&lt;=0.005,"OK","CHECK")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="B19" s="74" t="n">
-        <f aca="false">Comps!D31</f>
-        <v>8.66598514860548</v>
-      </c>
-      <c r="C19" s="73" t="n">
-        <v>8.66598</v>
       </c>
       <c r="D19" s="72" t="n">
         <f aca="false">B19-C19</f>
-        <v>5.14860547973228E-006</v>
+        <v>5.5676088621226E-005</v>
       </c>
       <c r="E19" s="12" t="str">
         <f aca="false">IF(ABS(D19)&lt;=0.005,"OK","CHECK")</f>
@@ -8389,30 +8398,50 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B20" s="74" t="n">
+        <f aca="false">Comps!D31</f>
+        <v>8.66598514860548</v>
+      </c>
+      <c r="C20" s="73" t="n">
+        <v>8.66598</v>
+      </c>
+      <c r="D20" s="72" t="n">
+        <f aca="false">B20-C20</f>
+        <v>5.14860547973228E-006</v>
+      </c>
+      <c r="E20" s="12" t="str">
+        <f aca="false">IF(ABS(D20)&lt;=0.005,"OK","CHECK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>493</v>
+      </c>
+      <c r="B21" s="74" t="n">
         <f aca="false">Assumptions!C5</f>
         <v>2</v>
       </c>
-      <c r="C20" s="73" t="n">
+      <c r="C21" s="73" t="n">
         <v>2</v>
       </c>
-      <c r="D20" s="72" t="n">
-        <f aca="false">B20-C20</f>
+      <c r="D21" s="72" t="n">
+        <f aca="false">B21-C21</f>
         <v>0</v>
       </c>
-      <c r="E20" s="12" t="str">
-        <f aca="false">IF(ABS(D20)&lt;=0,"OK","CHECK")</f>
+      <c r="E21" s="12" t="str">
+        <f aca="false">IF(ABS(D21)&lt;=0,"OK","CHECK")</f>
         <v>OK</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12" t="s">
-        <v>491</v>
-      </c>
-      <c r="E22" s="75" t="str">
-        <f aca="false">IF(COUNTIF(E6:E20,"OK")=15,"ALL OK","REVIEW")</f>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="12" t="s">
+        <v>494</v>
+      </c>
+      <c r="E23" s="75" t="str">
+        <f aca="false">IF(COUNTIF(E6:E21,"OK")=16,"ALL OK","REVIEW")</f>
         <v>ALL OK</v>
       </c>
     </row>
@@ -14663,7 +14692,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="60"/>
@@ -15351,9 +15380,9 @@
       <c r="A52" s="6" t="s">
         <v>385</v>
       </c>
-      <c r="B52" s="23" t="n">
-        <f aca="false">B42+B43-B44-B45</f>
-        <v>4487</v>
+      <c r="B52" s="53" t="n">
+        <f aca="false">B35*(1+$B$8)^0.5/G29</f>
+        <v>10.3234520203114</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15361,28 +15390,46 @@
         <v>386</v>
       </c>
       <c r="B53" s="23" t="n">
-        <f aca="false">WACC!$B$21-B52</f>
-        <v>431365.4563756</v>
+        <f aca="false">B42+B43-B44-B45</f>
+        <v>4487</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="B54" s="53" t="n">
-        <f aca="false">B53/C29</f>
-        <v>34.1655599491446</v>
+      <c r="B54" s="23" t="n">
+        <f aca="false">WACC!$B$21-B53</f>
+        <v>431365.4563756</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="6" t="s">
         <v>388</v>
       </c>
-      <c r="B55" s="29" t="n">
+      <c r="B55" s="53" t="n">
+        <f aca="false">B54/G29</f>
+        <v>26.0731527578601</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="6" t="s">
+        <v>389</v>
+      </c>
+      <c r="B56" s="53" t="n">
+        <f aca="false">B54/C29</f>
+        <v>34.1655599491446</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="B57" s="29" t="n">
         <v>0.070525</v>
       </c>
-      <c r="C55" s="3" t="s">
-        <v>389</v>
+      <c r="C57" s="3" t="s">
+        <v>391</v>
       </c>
     </row>
   </sheetData>
@@ -15410,7 +15457,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15420,22 +15467,22 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="40" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15461,23 +15508,23 @@
         <v>0.0738248058531887</v>
       </c>
       <c r="B10" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A10)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$9)*(1-DCF!$B$11)*(1-B$9/DCF!$B$10)/($A10-B$9)/(1+$A10)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A10)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$9)*(1-DCF!$B$11)*(1-B$9/DCF!$B$10)/($A10-B$9)/(1+$A10)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>357.903999636959</v>
       </c>
       <c r="C10" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A10)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$9)*(1-DCF!$B$11)*(1-C$9/DCF!$B$10)/($A10-C$9)/(1+$A10)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A10)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$9)*(1-DCF!$B$11)*(1-C$9/DCF!$B$10)/($A10-C$9)/(1+$A10)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>381.800040582807</v>
       </c>
       <c r="D10" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A10)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$9)*(1-DCF!$B$11)*(1-D$9/DCF!$B$10)/($A10-D$9)/(1+$A10)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A10)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$9)*(1-DCF!$B$11)*(1-D$9/DCF!$B$10)/($A10-D$9)/(1+$A10)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>411.074003914822</v>
       </c>
       <c r="E10" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A10)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$9)*(1-DCF!$B$11)*(1-E$9/DCF!$B$10)/($A10-E$9)/(1+$A10)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A10)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$9)*(1-DCF!$B$11)*(1-E$9/DCF!$B$10)/($A10-E$9)/(1+$A10)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>447.803654969361</v>
       </c>
       <c r="F10" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A10)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$9)*(1-DCF!$B$11)*(1-F$9/DCF!$B$10)/($A10-F$9)/(1+$A10)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A10)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$9)*(1-DCF!$B$11)*(1-F$9/DCF!$B$10)/($A10-F$9)/(1+$A10)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>495.295304396757</v>
       </c>
     </row>
@@ -15487,23 +15534,23 @@
         <v>0.0788248058531887</v>
       </c>
       <c r="B11" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A11)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$9)*(1-DCF!$B$11)*(1-B$9/DCF!$B$10)/($A11-B$9)/(1+$A11)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A11)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$9)*(1-DCF!$B$11)*(1-B$9/DCF!$B$10)/($A11-B$9)/(1+$A11)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>328.108546726339</v>
       </c>
       <c r="C11" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A11)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$9)*(1-DCF!$B$11)*(1-C$9/DCF!$B$10)/($A11-C$9)/(1+$A11)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A11)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$9)*(1-DCF!$B$11)*(1-C$9/DCF!$B$10)/($A11-C$9)/(1+$A11)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>347.165983784798</v>
       </c>
       <c r="D11" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A11)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$9)*(1-DCF!$B$11)*(1-D$9/DCF!$B$10)/($A11-D$9)/(1+$A11)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A11)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$9)*(1-DCF!$B$11)*(1-D$9/DCF!$B$10)/($A11-D$9)/(1+$A11)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>370.060854400481</v>
       </c>
       <c r="E11" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A11)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$9)*(1-DCF!$B$11)*(1-E$9/DCF!$B$10)/($A11-E$9)/(1+$A11)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A11)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$9)*(1-DCF!$B$11)*(1-E$9/DCF!$B$10)/($A11-E$9)/(1+$A11)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>398.106604286104</v>
       </c>
       <c r="F11" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A11)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$9)*(1-DCF!$B$11)*(1-F$9/DCF!$B$10)/($A11-F$9)/(1+$A11)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A11)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$9)*(1-DCF!$B$11)*(1-F$9/DCF!$B$10)/($A11-F$9)/(1+$A11)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>433.293280458029</v>
       </c>
     </row>
@@ -15513,23 +15560,23 @@
         <v>0.0838248058531887</v>
       </c>
       <c r="B12" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A12)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$9)*(1-DCF!$B$11)*(1-B$9/DCF!$B$10)/($A12-B$9)/(1+$A12)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A12)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$9)*(1-DCF!$B$11)*(1-B$9/DCF!$B$10)/($A12-B$9)/(1+$A12)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>303.000483449761</v>
       </c>
       <c r="C12" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A12)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$9)*(1-DCF!$B$11)*(1-C$9/DCF!$B$10)/($A12-C$9)/(1+$A12)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A12)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$9)*(1-DCF!$B$11)*(1-C$9/DCF!$B$10)/($A12-C$9)/(1+$A12)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>318.437365126815</v>
       </c>
       <c r="D12" s="57" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A12)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$9)*(1-DCF!$B$11)*(1-D$9/DCF!$B$10)/($A12-D$9)/(1+$A12)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A12)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$9)*(1-DCF!$B$11)*(1-D$9/DCF!$B$10)/($A12-D$9)/(1+$A12)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>336.683667848478</v>
       </c>
       <c r="E12" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A12)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$9)*(1-DCF!$B$11)*(1-E$9/DCF!$B$10)/($A12-E$9)/(1+$A12)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A12)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$9)*(1-DCF!$B$11)*(1-E$9/DCF!$B$10)/($A12-E$9)/(1+$A12)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>358.602504430718</v>
       </c>
       <c r="F12" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A12)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$9)*(1-DCF!$B$11)*(1-F$9/DCF!$B$10)/($A12-F$9)/(1+$A12)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A12)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$9)*(1-DCF!$B$11)*(1-F$9/DCF!$B$10)/($A12-F$9)/(1+$A12)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>385.450880052138</v>
       </c>
     </row>
@@ -15539,23 +15586,23 @@
         <v>0.0888248058531887</v>
       </c>
       <c r="B13" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A13)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$9)*(1-DCF!$B$11)*(1-B$9/DCF!$B$10)/($A13-B$9)/(1+$A13)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A13)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$9)*(1-DCF!$B$11)*(1-B$9/DCF!$B$10)/($A13-B$9)/(1+$A13)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>281.557728421472</v>
       </c>
       <c r="C13" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A13)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$9)*(1-DCF!$B$11)*(1-C$9/DCF!$B$10)/($A13-C$9)/(1+$A13)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A13)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$9)*(1-DCF!$B$11)*(1-C$9/DCF!$B$10)/($A13-C$9)/(1+$A13)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>294.22584153849</v>
       </c>
       <c r="D13" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A13)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$9)*(1-DCF!$B$11)*(1-D$9/DCF!$B$10)/($A13-D$9)/(1+$A13)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A13)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$9)*(1-DCF!$B$11)*(1-D$9/DCF!$B$10)/($A13-D$9)/(1+$A13)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>308.994898420695</v>
       </c>
       <c r="E13" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A13)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$9)*(1-DCF!$B$11)*(1-E$9/DCF!$B$10)/($A13-E$9)/(1+$A13)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A13)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$9)*(1-DCF!$B$11)*(1-E$9/DCF!$B$10)/($A13-E$9)/(1+$A13)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>326.450394101058</v>
       </c>
       <c r="F13" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A13)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$9)*(1-DCF!$B$11)*(1-F$9/DCF!$B$10)/($A13-F$9)/(1+$A13)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A13)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$9)*(1-DCF!$B$11)*(1-F$9/DCF!$B$10)/($A13-F$9)/(1+$A13)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>347.417658681118</v>
       </c>
     </row>
@@ -15565,34 +15612,34 @@
         <v>0.0938248058531887</v>
       </c>
       <c r="B14" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A14)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$9)*(1-DCF!$B$11)*(1-B$9/DCF!$B$10)/($A14-B$9)/(1+$A14)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A14)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$9)*(1-DCF!$B$11)*(1-B$9/DCF!$B$10)/($A14-B$9)/(1+$A14)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>263.035108449863</v>
       </c>
       <c r="C14" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A14)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$9)*(1-DCF!$B$11)*(1-C$9/DCF!$B$10)/($A14-C$9)/(1+$A14)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A14)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$9)*(1-DCF!$B$11)*(1-C$9/DCF!$B$10)/($A14-C$9)/(1+$A14)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>273.546526007043</v>
       </c>
       <c r="D14" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A14)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$9)*(1-DCF!$B$11)*(1-D$9/DCF!$B$10)/($A14-D$9)/(1+$A14)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A14)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$9)*(1-DCF!$B$11)*(1-D$9/DCF!$B$10)/($A14-D$9)/(1+$A14)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>285.657291150351</v>
       </c>
       <c r="E14" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A14)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$9)*(1-DCF!$B$11)*(1-E$9/DCF!$B$10)/($A14-E$9)/(1+$A14)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A14)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$9)*(1-DCF!$B$11)*(1-E$9/DCF!$B$10)/($A14-E$9)/(1+$A14)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>299.775228664656</v>
       </c>
       <c r="F14" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A14)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$9)*(1-DCF!$B$11)*(1-F$9/DCF!$B$10)/($A14-F$9)/(1+$A14)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+$A14)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$9)*(1-DCF!$B$11)*(1-F$9/DCF!$B$10)/($A14-F$9)/(1+$A14)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>316.459701191172</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="40" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15617,23 +15664,23 @@
         <v>0.15</v>
       </c>
       <c r="B19" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$18)*(1-DCF!$B$11)*(1-B$18/$A19)/(DCF!$B$8-B$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$18)*(1-DCF!$B$11)*(1-B$18/$A19)/(DCF!$B$8-B$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>289.566542705876</v>
       </c>
       <c r="C19" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$18)*(1-DCF!$B$11)*(1-C$18/$A19)/(DCF!$B$8-C$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$18)*(1-DCF!$B$11)*(1-C$18/$A19)/(DCF!$B$8-C$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>300.128301459476</v>
       </c>
       <c r="D19" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$18)*(1-DCF!$B$11)*(1-D$18/$A19)/(DCF!$B$8-D$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$18)*(1-DCF!$B$11)*(1-D$18/$A19)/(DCF!$B$8-D$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>312.554698554774</v>
       </c>
       <c r="E19" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$18)*(1-DCF!$B$11)*(1-E$18/$A19)/(DCF!$B$8-E$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$18)*(1-DCF!$B$11)*(1-E$18/$A19)/(DCF!$B$8-E$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>327.418589830859</v>
       </c>
       <c r="F19" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$18)*(1-DCF!$B$11)*(1-F$18/$A19)/(DCF!$B$8-F$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$18)*(1-DCF!$B$11)*(1-F$18/$A19)/(DCF!$B$8-F$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>345.554261076341</v>
       </c>
     </row>
@@ -15642,23 +15689,23 @@
         <v>0.2</v>
       </c>
       <c r="B20" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$18)*(1-DCF!$B$11)*(1-B$18/$A20)/(DCF!$B$8-B$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$18)*(1-DCF!$B$11)*(1-B$18/$A20)/(DCF!$B$8-B$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>297.962755670804</v>
       </c>
       <c r="C20" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$18)*(1-DCF!$B$11)*(1-C$18/$A20)/(DCF!$B$8-C$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$18)*(1-DCF!$B$11)*(1-C$18/$A20)/(DCF!$B$8-C$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>311.571466251563</v>
       </c>
       <c r="D20" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$18)*(1-DCF!$B$11)*(1-D$18/$A20)/(DCF!$B$8-D$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$18)*(1-DCF!$B$11)*(1-D$18/$A20)/(DCF!$B$8-D$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>327.635304363339</v>
       </c>
       <c r="E20" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$18)*(1-DCF!$B$11)*(1-E$18/$A20)/(DCF!$B$8-E$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$18)*(1-DCF!$B$11)*(1-E$18/$A20)/(DCF!$B$8-E$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>346.908536455771</v>
       </c>
       <c r="F20" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$18)*(1-DCF!$B$11)*(1-F$18/$A20)/(DCF!$B$8-F$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$18)*(1-DCF!$B$11)*(1-F$18/$A20)/(DCF!$B$8-F$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>370.489647936214</v>
       </c>
     </row>
@@ -15667,23 +15714,23 @@
         <v>0.25</v>
       </c>
       <c r="B21" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$18)*(1-DCF!$B$11)*(1-B$18/$A21)/(DCF!$B$8-B$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$18)*(1-DCF!$B$11)*(1-B$18/$A21)/(DCF!$B$8-B$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>303.000483449761</v>
       </c>
       <c r="C21" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$18)*(1-DCF!$B$11)*(1-C$18/$A21)/(DCF!$B$8-C$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$18)*(1-DCF!$B$11)*(1-C$18/$A21)/(DCF!$B$8-C$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>318.437365126815</v>
       </c>
       <c r="D21" s="57" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$18)*(1-DCF!$B$11)*(1-D$18/$A21)/(DCF!$B$8-D$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$18)*(1-DCF!$B$11)*(1-D$18/$A21)/(DCF!$B$8-D$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>336.683667848478</v>
       </c>
       <c r="E21" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$18)*(1-DCF!$B$11)*(1-E$18/$A21)/(DCF!$B$8-E$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$18)*(1-DCF!$B$11)*(1-E$18/$A21)/(DCF!$B$8-E$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>358.602504430718</v>
       </c>
       <c r="F21" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$18)*(1-DCF!$B$11)*(1-F$18/$A21)/(DCF!$B$8-F$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$18)*(1-DCF!$B$11)*(1-F$18/$A21)/(DCF!$B$8-F$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>385.450880052138</v>
       </c>
     </row>
@@ -15692,23 +15739,23 @@
         <v>0.3</v>
       </c>
       <c r="B22" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$18)*(1-DCF!$B$11)*(1-B$18/$A22)/(DCF!$B$8-B$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$18)*(1-DCF!$B$11)*(1-B$18/$A22)/(DCF!$B$8-B$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>306.358968635733</v>
       </c>
       <c r="C22" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$18)*(1-DCF!$B$11)*(1-C$18/$A22)/(DCF!$B$8-C$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$18)*(1-DCF!$B$11)*(1-C$18/$A22)/(DCF!$B$8-C$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>323.01463104365</v>
       </c>
       <c r="D22" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$18)*(1-DCF!$B$11)*(1-D$18/$A22)/(DCF!$B$8-D$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$18)*(1-DCF!$B$11)*(1-D$18/$A22)/(DCF!$B$8-D$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>342.715910171903</v>
       </c>
       <c r="E22" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$18)*(1-DCF!$B$11)*(1-E$18/$A22)/(DCF!$B$8-E$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$18)*(1-DCF!$B$11)*(1-E$18/$A22)/(DCF!$B$8-E$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>366.398483080682</v>
       </c>
       <c r="F22" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$18)*(1-DCF!$B$11)*(1-F$18/$A22)/(DCF!$B$8-F$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$18)*(1-DCF!$B$11)*(1-F$18/$A22)/(DCF!$B$8-F$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>395.425034796087</v>
       </c>
     </row>
@@ -15717,56 +15764,56 @@
         <v>0.35</v>
       </c>
       <c r="B23" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$18)*(1-DCF!$B$11)*(1-B$18/$A23)/(DCF!$B$8-B$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+B$18)*(1-DCF!$B$11)*(1-B$18/$A23)/(DCF!$B$8-B$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>308.757886625712</v>
       </c>
       <c r="C23" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$18)*(1-DCF!$B$11)*(1-C$18/$A23)/(DCF!$B$8-C$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+C$18)*(1-DCF!$B$11)*(1-C$18/$A23)/(DCF!$B$8-C$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>326.284106698532</v>
       </c>
       <c r="D23" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$18)*(1-DCF!$B$11)*(1-D$18/$A23)/(DCF!$B$8-D$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+D$18)*(1-DCF!$B$11)*(1-D$18/$A23)/(DCF!$B$8-D$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>347.024654688636</v>
       </c>
       <c r="E23" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$18)*(1-DCF!$B$11)*(1-E$18/$A23)/(DCF!$B$8-E$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+E$18)*(1-DCF!$B$11)*(1-E$18/$A23)/(DCF!$B$8-E$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>371.967039259229</v>
       </c>
       <c r="F23" s="56" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$18)*(1-DCF!$B$11)*(1-F$18/$A23)/(DCF!$B$8-F$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$52)/DCF!$B$47</f>
+        <f aca="false">(SUMPRODUCT(DCF!$C$26:$G$26,(1+DCF!$B$8)^(-DCF!$C$25:$G$25))+DCF!$G$15*(1+F$18)*(1-DCF!$B$11)*(1-F$18/$A23)/(DCF!$B$8-F$18)/(1+DCF!$B$8)^DCF!$G$25+DCF!$B$53)/DCF!$B$47</f>
         <v>402.549431041765</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="40" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="5" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B28" s="58" t="n">
         <v>298.921</v>
@@ -15786,7 +15833,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B29" s="58" t="n">
         <v>304.283</v>
@@ -15806,7 +15853,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B30" s="58" t="n">
         <v>309.857</v>
@@ -15826,7 +15873,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B31" s="58" t="n">
         <v>315.649</v>
@@ -15846,7 +15893,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B32" s="58" t="n">
         <v>321.666</v>
@@ -15866,24 +15913,24 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="40" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="16"/>
       <c r="B35" s="17" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="C35" s="17" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="D35" s="17" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B36" s="27" t="n">
         <v>0.0486635</v>
@@ -15897,7 +15944,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B37" s="29" t="n">
         <v>0.0356714</v>
@@ -15953,7 +16000,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B41" s="27" t="n">
         <v>0.25</v>
@@ -15967,7 +16014,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="12" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B42" s="60" t="n">
         <f aca="false">SUMPRODUCT(B40:D40,B41:D41)</f>
@@ -16001,7 +16048,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16011,7 +16058,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16020,33 +16067,33 @@
         <v>135</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="I5" s="17" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="C6" s="19" t="n">
         <v>979.88</v>
@@ -16072,7 +16119,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>193</v>
@@ -16101,7 +16148,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>175</v>
@@ -16130,7 +16177,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>175</v>
@@ -16159,7 +16206,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>175</v>
@@ -16188,7 +16235,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>175</v>
@@ -16217,7 +16264,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>175</v>
@@ -16246,7 +16293,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>175</v>
@@ -16275,7 +16322,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>175</v>
@@ -16304,7 +16351,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>149</v>
@@ -16333,7 +16380,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>149</v>
@@ -16362,7 +16409,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="C18" s="61" t="n">
         <f aca="false">C6*C7</f>
@@ -16428,7 +16475,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C20" s="61" t="n">
         <f aca="false">C12+C13</f>
@@ -16461,7 +16508,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="C21" s="62" t="n">
         <f aca="false">C20/C11</f>
@@ -16494,7 +16541,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="C22" s="63" t="n">
         <f aca="false">C19/C11</f>
@@ -16527,7 +16574,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="C23" s="64" t="n">
         <f aca="false">IF(C20&gt;0,C19/C20,"NM")</f>
@@ -16560,7 +16607,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="C24" s="64" t="n">
         <f aca="false">IF(C14&gt;0,C18/C14,"NM")</f>
@@ -16593,7 +16640,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="C25" s="63" t="n">
         <f aca="false">C18/C11</f>
@@ -16626,7 +16673,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="C26" s="65" t="n">
         <f aca="false">IF(ISNUMBER(C23),C23/(C16*100),"NM")</f>
@@ -16659,57 +16706,57 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="C27" s="66" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="D27" s="66" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="E27" s="66" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="F27" s="66" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="G27" s="66" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="H27" s="66" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="I27" s="66" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="16" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B29" s="17"/>
       <c r="C29" s="17" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="D29" s="17" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="E29" s="17" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="F29" s="17" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="G29" s="17" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="H29" s="17" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="C30" s="53" t="n">
         <f aca="false">QUARTILE(D22:I22,1)</f>
@@ -16738,7 +16785,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="C31" s="53" t="n">
         <f aca="false">QUARTILE(D23:I23,1)</f>
@@ -16767,7 +16814,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="C32" s="53" t="n">
         <f aca="false">QUARTILE(D24:I24,1)</f>
@@ -16796,7 +16843,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="C33" s="53" t="n">
         <f aca="false">QUARTILE(D25:I25,1)</f>
@@ -16825,7 +16872,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="C34" s="53" t="n">
         <f aca="false">QUARTILE(D26:I26,1)</f>
@@ -16854,27 +16901,27 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="16" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="C36" s="17" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="D36" s="17" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="E36" s="17" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="F36" s="17" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B37" s="23" t="n">
         <f aca="false">C20</f>
@@ -16899,7 +16946,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B38" s="23" t="n">
         <f aca="false">C11</f>
@@ -16924,7 +16971,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B39" s="23" t="n">
         <f aca="false">C14</f>
@@ -16949,7 +16996,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B40" s="23" t="n">
         <f aca="false">C11</f>

</xml_diff>

<commit_message>
Add PriceSmart (PSMT) to Tier 1 comps (review 3e)
- Config: PSMT (CIK 1041803) in settings.json and peers.json (Tier 1)
- sec_fetch: --only option to add a company without re-downloading everything
- Market data: PSMT daily and monthly prices (Yahoo, checksum-verified, in manifest)
- Comps: PSMT 8.9x EV/EBITDA, 20.3x P/E. Tier 1 median now BJ's (13.2x / 23.9x);
  selected range ~$360-$690 (was ~$450-$690). Peer median 8.8x / 18.4x
- Peer-beta WACC cross-check 7.50% / $400 (was 7.23% / $425); DCF unchanged at $337
- Excel Comps sheet handles any number of peers, adds Walmart column and a check;
  Summary uses the selected range. Charts 12 and 14, memo, deck, README, docs updated
</commit_message>
<xml_diff>
--- a/outputs/COST_Valuation_Model.xlsx
+++ b/outputs/COST_Valuation_Model.xlsx
@@ -5419,12 +5419,36 @@
         </r>
       </text>
     </comment>
+    <comment ref="J8" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Balance sheet 2024-11-30; finance leases: not tagged</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">LTM to 2024-11-30 (fiscal year + YTD - prior YTD), scaled to 52 weeks</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="495">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="498">
   <si>
     <t xml:space="preserve">Costco Wholesale Corporation (COST): Equity Research and Valuation Model</t>
   </si>
@@ -6710,6 +6734,9 @@
     <t xml:space="preserve">KR</t>
   </si>
   <si>
+    <t xml:space="preserve">PSMT</t>
+  </si>
+  <si>
     <t xml:space="preserve">Share price 31 Jan 2025</t>
   </si>
   <si>
@@ -6806,6 +6833,9 @@
     <t xml:space="preserve">vs. median</t>
   </si>
   <si>
+    <t xml:space="preserve">Walmart</t>
+  </si>
+  <si>
     <t xml:space="preserve">Implied Costco value per share ($)</t>
   </si>
   <si>
@@ -6845,7 +6875,7 @@
     <t xml:space="preserve">Comps: EV/Revenue (peer 25th-75th)</t>
   </si>
   <si>
-    <t xml:space="preserve">Comps: Tier 1 median (EV/EBITDA to P/E)</t>
+    <t xml:space="preserve">Comps selected range: Tier 1 median EV/EBITDA to Walmart P/E</t>
   </si>
   <si>
     <t xml:space="preserve">Share price, 31 Jan 2025</t>
@@ -6903,6 +6933,9 @@
   </si>
   <si>
     <t xml:space="preserve">Comps: peer median EV/EBITDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comps: selected range, Walmart P/E implied value ($)</t>
   </si>
   <si>
     <t xml:space="preserve">Scenario selector is on Base (2)</t>
@@ -7748,7 +7781,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="7" t="str">
-        <f aca="false">Checks!E23</f>
+        <f aca="false">Checks!E24</f>
         <v>ALL OK</v>
       </c>
     </row>
@@ -7906,7 +7939,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7916,26 +7949,26 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B6" s="68" t="n">
         <f aca="false">Sensitivity!B40</f>
@@ -7952,7 +7985,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B7" s="56" t="n">
         <f aca="false">MIN(Sensitivity!C11:E13)</f>
@@ -7969,71 +8002,71 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B8" s="68" t="n">
         <f aca="false">Comps!C37</f>
-        <v>208.422465418063</v>
+        <v>216.34231151994</v>
       </c>
       <c r="C8" s="68" t="n">
         <f aca="false">Comps!D37</f>
-        <v>240.101849825571</v>
+        <v>242.819693575233</v>
       </c>
       <c r="D8" s="68" t="n">
         <f aca="false">Comps!E37</f>
-        <v>359.34629792755</v>
+        <v>330.894107776887</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B9" s="68" t="n">
         <f aca="false">Comps!C39</f>
-        <v>251.54102063944</v>
+        <v>258.756788605664</v>
       </c>
       <c r="C9" s="68" t="n">
         <f aca="false">Comps!D39</f>
-        <v>280.404092504339</v>
+        <v>313.312330776693</v>
       </c>
       <c r="D9" s="68" t="n">
         <f aca="false">Comps!E39</f>
-        <v>408.151966254981</v>
+        <v>392.669116953498</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B10" s="68" t="n">
         <f aca="false">Comps!C38</f>
-        <v>330.409661486618</v>
+        <v>322.494784853975</v>
       </c>
       <c r="C10" s="68" t="n">
         <f aca="false">Comps!D38</f>
-        <v>384.42207834136</v>
+        <v>362.344418777918</v>
       </c>
       <c r="D10" s="68" t="n">
         <f aca="false">Comps!E38</f>
-        <v>423.009756092804</v>
+        <v>417.506416696804</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B11" s="68" t="n">
         <f aca="false">Comps!F37</f>
-        <v>452.488830752367</v>
+        <v>359.34629792755</v>
       </c>
       <c r="D11" s="68" t="n">
-        <f aca="false">Comps!F39</f>
-        <v>547.951826169626</v>
+        <f aca="false">Comps!G39</f>
+        <v>687.751686084271</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="C13" s="69" t="n">
         <f aca="false">DCF!B49</f>
@@ -8042,7 +8075,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="C14" s="70" t="n">
         <f aca="false">Sensitivity!B42</f>
@@ -8051,7 +8084,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="C15" s="71" t="n">
         <f aca="false">DCF!B50</f>
@@ -8074,7 +8107,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
@@ -8096,29 +8129,29 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B6" s="72" t="n">
         <f aca="false">SUMPRODUCT(ABS(Forecast!C54:H54))</f>
@@ -8138,7 +8171,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B7" s="72" t="n">
         <f aca="false">SUMPRODUCT(ABS(Forecast!D33:H33-Forecast!C33:G33-Forecast!D67:H67))</f>
@@ -8158,7 +8191,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B8" s="74" t="n">
         <f aca="false">Forecast!C18</f>
@@ -8178,7 +8211,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B9" s="74" t="n">
         <f aca="false">Forecast!H18</f>
@@ -8198,7 +8231,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B10" s="74" t="n">
         <f aca="false">Forecast!H21</f>
@@ -8218,7 +8251,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B11" s="74" t="n">
         <f aca="false">Forecast!D28</f>
@@ -8338,7 +8371,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B17" s="74" t="n">
         <f aca="false">DCF!B52</f>
@@ -8358,7 +8391,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B18" s="74" t="n">
         <f aca="false">Sensitivity!D12</f>
@@ -8378,7 +8411,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B19" s="74" t="n">
         <f aca="false">Comps!G31</f>
@@ -8398,18 +8431,18 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B20" s="74" t="n">
         <f aca="false">Comps!D31</f>
-        <v>8.66598514860548</v>
+        <v>8.76839140636215</v>
       </c>
       <c r="C20" s="73" t="n">
-        <v>8.66598</v>
+        <v>8.76839</v>
       </c>
       <c r="D20" s="72" t="n">
         <f aca="false">B20-C20</f>
-        <v>5.14860547973228E-006</v>
+        <v>1.40636215384404E-006</v>
       </c>
       <c r="E20" s="12" t="str">
         <f aca="false">IF(ABS(D20)&lt;=0.005,"OK","CHECK")</f>
@@ -8418,30 +8451,50 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B21" s="74" t="n">
+        <f aca="false">Comps!G39</f>
+        <v>687.751686084271</v>
+      </c>
+      <c r="C21" s="73" t="n">
+        <v>687.752</v>
+      </c>
+      <c r="D21" s="72" t="n">
+        <f aca="false">B21-C21</f>
+        <v>-0.000313915729179826</v>
+      </c>
+      <c r="E21" s="12" t="str">
+        <f aca="false">IF(ABS(D21)&lt;=0.05,"OK","CHECK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="B22" s="74" t="n">
         <f aca="false">Assumptions!C5</f>
         <v>2</v>
       </c>
-      <c r="C21" s="73" t="n">
+      <c r="C22" s="73" t="n">
         <v>2</v>
       </c>
-      <c r="D21" s="72" t="n">
-        <f aca="false">B21-C21</f>
+      <c r="D22" s="72" t="n">
+        <f aca="false">B22-C22</f>
         <v>0</v>
       </c>
-      <c r="E21" s="12" t="str">
-        <f aca="false">IF(ABS(D21)&lt;=0,"OK","CHECK")</f>
+      <c r="E22" s="12" t="str">
+        <f aca="false">IF(ABS(D22)&lt;=0,"OK","CHECK")</f>
         <v>OK</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12" t="s">
-        <v>494</v>
-      </c>
-      <c r="E23" s="75" t="str">
-        <f aca="false">IF(COUNTIF(E6:E21,"OK")=16,"ALL OK","REVIEW")</f>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="12" t="s">
+        <v>497</v>
+      </c>
+      <c r="E24" s="75" t="str">
+        <f aca="false">IF(COUNTIF(E6:E22,"OK")=17,"ALL OK","REVIEW")</f>
         <v>ALL OK</v>
       </c>
     </row>
@@ -16037,13 +16090,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="3" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16087,13 +16140,16 @@
       <c r="I5" s="17" t="s">
         <v>427</v>
       </c>
+      <c r="J5" s="17" t="s">
+        <v>428</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C6" s="19" t="n">
         <v>979.88</v>
@@ -16116,10 +16172,13 @@
       <c r="I6" s="19" t="n">
         <v>61.64</v>
       </c>
+      <c r="J6" s="19" t="n">
+        <v>90.97</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>193</v>
@@ -16145,10 +16204,13 @@
       <c r="I7" s="20" t="n">
         <v>723.606</v>
       </c>
+      <c r="J7" s="20" t="n">
+        <v>30.6623</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>175</v>
@@ -16174,10 +16236,13 @@
       <c r="I8" s="18" t="n">
         <v>22617</v>
       </c>
+      <c r="J8" s="18" t="n">
+        <v>123.386</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>175</v>
@@ -16203,10 +16268,13 @@
       <c r="I9" s="18" t="n">
         <v>-6</v>
       </c>
+      <c r="J9" s="18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>175</v>
@@ -16232,10 +16300,13 @@
       <c r="I10" s="18" t="n">
         <v>13358</v>
       </c>
+      <c r="J10" s="18" t="n">
+        <v>222.195</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>175</v>
@@ -16261,10 +16332,13 @@
       <c r="I11" s="18" t="n">
         <v>147051</v>
       </c>
+      <c r="J11" s="18" t="n">
+        <v>4978.02</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>175</v>
@@ -16290,10 +16364,13 @@
       <c r="I12" s="18" t="n">
         <v>4053.06</v>
       </c>
+      <c r="J12" s="18" t="n">
+        <v>219.783</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>175</v>
@@ -16319,10 +16396,13 @@
       <c r="I13" s="18" t="n">
         <v>3154.34</v>
       </c>
+      <c r="J13" s="18" t="n">
+        <v>83.5201</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>175</v>
@@ -16348,10 +16428,13 @@
       <c r="I14" s="18" t="n">
         <v>2714.79</v>
       </c>
+      <c r="J14" s="18" t="n">
+        <v>137.501</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>149</v>
@@ -16377,10 +16460,13 @@
       <c r="I15" s="27" t="n">
         <v>-0.00141624</v>
       </c>
+      <c r="J15" s="27" t="n">
+        <v>0.0784149</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>149</v>
@@ -16406,10 +16492,13 @@
       <c r="I16" s="27" t="n">
         <v>0.0357162</v>
       </c>
+      <c r="J16" s="27" t="n">
+        <v>0.106237</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C18" s="61" t="n">
         <f aca="false">C6*C7</f>
@@ -16439,6 +16528,10 @@
         <f aca="false">I6*I7</f>
         <v>44603.07384</v>
       </c>
+      <c r="J18" s="61" t="n">
+        <f aca="false">J6*J7</f>
+        <v>2789.349431</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
@@ -16472,10 +16565,14 @@
         <f aca="false">I18+I8+I9-I10</f>
         <v>53856.07384</v>
       </c>
+      <c r="J19" s="61" t="n">
+        <f aca="false">J18+J8+J9-J10</f>
+        <v>2690.540431</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C20" s="61" t="n">
         <f aca="false">C12+C13</f>
@@ -16505,10 +16602,14 @@
         <f aca="false">I12+I13</f>
         <v>7207.4</v>
       </c>
+      <c r="J20" s="61" t="n">
+        <f aca="false">J12+J13</f>
+        <v>303.3031</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C21" s="62" t="n">
         <f aca="false">C20/C11</f>
@@ -16538,10 +16639,14 @@
         <f aca="false">I20/I11</f>
         <v>0.0490129274877423</v>
       </c>
+      <c r="J21" s="62" t="n">
+        <f aca="false">J20/J11</f>
+        <v>0.060928461516828</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C22" s="63" t="n">
         <f aca="false">C19/C11</f>
@@ -16571,10 +16676,14 @@
         <f aca="false">I19/I11</f>
         <v>0.366240786121822</v>
       </c>
+      <c r="J22" s="63" t="n">
+        <f aca="false">J19/J11</f>
+        <v>0.540484054101832</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C23" s="64" t="n">
         <f aca="false">IF(C20&gt;0,C19/C20,"NM")</f>
@@ -16604,10 +16713,14 @@
         <f aca="false">IF(I20&gt;0,I19/I20,"NM")</f>
         <v>7.47233036046286</v>
       </c>
+      <c r="J23" s="64" t="n">
+        <f aca="false">IF(J20&gt;0,J19/J20,"NM")</f>
+        <v>8.87079766411883</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C24" s="64" t="n">
         <f aca="false">IF(C14&gt;0,C18/C14,"NM")</f>
@@ -16637,10 +16750,14 @@
         <f aca="false">IF(I14&gt;0,I18/I14,"NM")</f>
         <v>16.4296589570464</v>
       </c>
+      <c r="J24" s="64" t="n">
+        <f aca="false">IF(J14&gt;0,J18/J14,"NM")</f>
+        <v>20.2860301452353</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C25" s="63" t="n">
         <f aca="false">C18/C11</f>
@@ -16670,10 +16787,14 @@
         <f aca="false">I18/I11</f>
         <v>0.303317038578452</v>
       </c>
+      <c r="J25" s="63" t="n">
+        <f aca="false">J18/J11</f>
+        <v>0.560333110553995</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C26" s="65" t="n">
         <f aca="false">IF(ISNUMBER(C23),C23/(C16*100),"NM")</f>
@@ -16703,76 +16824,86 @@
         <f aca="false">IF(ISNUMBER(I23),I23/(I16*100),"NM")</f>
         <v>2.09214036220619</v>
       </c>
+      <c r="J26" s="65" t="n">
+        <f aca="false">IF(ISNUMBER(J23),J23/(J16*100),"NM")</f>
+        <v>0.835000768481681</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C27" s="66" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D27" s="66" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E27" s="66" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="F27" s="66" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="G27" s="66" t="s">
+        <v>453</v>
+      </c>
+      <c r="H27" s="66" t="s">
+        <v>453</v>
+      </c>
+      <c r="I27" s="66" t="s">
         <v>452</v>
       </c>
-      <c r="H27" s="66" t="s">
-        <v>452</v>
-      </c>
-      <c r="I27" s="66" t="s">
+      <c r="J27" s="66" t="s">
         <v>451</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="16" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B29" s="17"/>
       <c r="C29" s="17" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D29" s="17" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="E29" s="17" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="F29" s="17" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="G29" s="17" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="H29" s="17" t="s">
-        <v>459</v>
+        <v>460</v>
+      </c>
+      <c r="I29" s="17" t="s">
+        <v>461</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C30" s="53" t="n">
-        <f aca="false">QUARTILE(D22:I22,1)</f>
-        <v>0.549377014834521</v>
+        <f aca="false">QUARTILE(D22:J22,1)</f>
+        <v>0.53580152045708</v>
       </c>
       <c r="D30" s="67" t="n">
-        <f aca="false">MEDIAN(D22:I22)</f>
-        <v>0.642018416002981</v>
+        <f aca="false">MEDIAN(D22:J22)</f>
+        <v>0.604151098901099</v>
       </c>
       <c r="E30" s="53" t="n">
-        <f aca="false">QUARTILE(D22:I22,3)</f>
-        <v>0.708203503486562</v>
+        <f aca="false">QUARTILE(D22:J22,3)</f>
+        <v>0.698764246692662</v>
       </c>
       <c r="F30" s="53" t="n">
-        <f aca="false">MEDIAN(D22,E22)</f>
-        <v>0.960705160232679</v>
+        <f aca="false">MEDIAN(D22,E22,J22)</f>
+        <v>0.679885733104862</v>
       </c>
       <c r="G30" s="53" t="n">
         <f aca="false">C22</f>
@@ -16780,28 +16911,32 @@
       </c>
       <c r="H30" s="21" t="n">
         <f aca="false">G30/D30-1</f>
-        <v>1.59079821748194</v>
+        <v>1.7531857027101</v>
+      </c>
+      <c r="I30" s="53" t="n">
+        <f aca="false">D22</f>
+        <v>1.2415245873605</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C31" s="53" t="n">
-        <f aca="false">QUARTILE(D23:I23,1)</f>
-        <v>7.47233036046286</v>
+        <f aca="false">QUARTILE(D23:J23,1)</f>
+        <v>7.77074405749851</v>
       </c>
       <c r="D31" s="67" t="n">
-        <f aca="false">MEDIAN(D23:I23)</f>
-        <v>8.66598514860548</v>
+        <f aca="false">MEDIAN(D23:J23)</f>
+        <v>8.76839140636215</v>
       </c>
       <c r="E31" s="53" t="n">
-        <f aca="false">QUARTILE(D23:I23,3)</f>
+        <f aca="false">QUARTILE(D23:J23,3)</f>
+        <v>12.0869674516639</v>
+      </c>
+      <c r="F31" s="53" t="n">
+        <f aca="false">MEDIAN(D23,E23,J23)</f>
         <v>13.1590240475122</v>
-      </c>
-      <c r="F31" s="53" t="n">
-        <f aca="false">MEDIAN(D23,E23)</f>
-        <v>16.6685628963709</v>
       </c>
       <c r="G31" s="53" t="n">
         <f aca="false">C23</f>
@@ -16809,28 +16944,32 @@
       </c>
       <c r="H31" s="21" t="n">
         <f aca="false">G31/D31-1</f>
-        <v>3.21651492005714</v>
+        <v>3.16727013914728</v>
+      </c>
+      <c r="I31" s="53" t="n">
+        <f aca="false">D23</f>
+        <v>20.1781017452295</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C32" s="53" t="n">
-        <f aca="false">QUARTILE(D24:I24,1)</f>
-        <v>14.7384909610384</v>
+        <f aca="false">QUARTILE(D24:J24,1)</f>
+        <v>15.1612829600404</v>
       </c>
       <c r="D32" s="67" t="n">
-        <f aca="false">MEDIAN(D24:I24)</f>
-        <v>16.4296589570464</v>
+        <f aca="false">MEDIAN(D24:J24)</f>
+        <v>18.3578445511409</v>
       </c>
       <c r="E32" s="53" t="n">
-        <f aca="false">QUARTILE(D24:I24,3)</f>
+        <f aca="false">QUARTILE(D24:J24,3)</f>
+        <v>23.0075802991738</v>
+      </c>
+      <c r="F32" s="53" t="n">
+        <f aca="false">MEDIAN(D24,E24,J24)</f>
         <v>23.91476368382</v>
-      </c>
-      <c r="F32" s="53" t="n">
-        <f aca="false">MEDIAN(D24,E24)</f>
-        <v>32.1060279415088</v>
       </c>
       <c r="G32" s="53" t="n">
         <f aca="false">C24</f>
@@ -16838,28 +16977,32 @@
       </c>
       <c r="H32" s="21" t="n">
         <f aca="false">G32/D32-1</f>
-        <v>2.49452816914517</v>
+        <v>2.12748622938301</v>
+      </c>
+      <c r="I32" s="53" t="n">
+        <f aca="false">D24</f>
+        <v>40.2972921991977</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C33" s="53" t="n">
-        <f aca="false">QUARTILE(D25:I25,1)</f>
-        <v>0.420547247801207</v>
+        <f aca="false">QUARTILE(D25:J25,1)</f>
+        <v>0.45201356058973</v>
       </c>
       <c r="D33" s="67" t="n">
-        <f aca="false">MEDIAN(D25:I25)</f>
-        <v>0.556847817927048</v>
+        <f aca="false">MEDIAN(D25:J25)</f>
+        <v>0.560333110553995</v>
       </c>
       <c r="E33" s="53" t="n">
-        <f aca="false">QUARTILE(D25:I25,3)</f>
-        <v>0.635663780296059</v>
+        <f aca="false">QUARTILE(D25:J25,3)</f>
+        <v>0.62335900342648</v>
       </c>
       <c r="F33" s="53" t="n">
-        <f aca="false">MEDIAN(D25,E25)</f>
-        <v>0.912339765893623</v>
+        <f aca="false">MEDIAN(D25,E25,J25)</f>
+        <v>0.647968557165638</v>
       </c>
       <c r="G33" s="53" t="n">
         <f aca="false">C25</f>
@@ -16867,28 +17010,32 @@
       </c>
       <c r="H33" s="21" t="n">
         <f aca="false">G33/D33-1</f>
-        <v>2.0181990325291</v>
+        <v>1.99942572315902</v>
+      </c>
+      <c r="I33" s="53" t="n">
+        <f aca="false">D25</f>
+        <v>1.17671097462161</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C34" s="53" t="n">
-        <f aca="false">QUARTILE(D26:I26,1)</f>
+        <f aca="false">QUARTILE(D26:J26,1)</f>
+        <v>1.56381856021545</v>
+      </c>
+      <c r="D34" s="67" t="n">
+        <f aca="false">MEDIAN(D26:J26)</f>
+        <v>1.84017167235721</v>
+      </c>
+      <c r="E34" s="53" t="n">
+        <f aca="false">QUARTILE(D26:J26,3)</f>
+        <v>2.12913997039411</v>
+      </c>
+      <c r="F34" s="53" t="n">
+        <f aca="false">MEDIAN(D26,E26,J26)</f>
         <v>1.58820298250822</v>
-      </c>
-      <c r="D34" s="67" t="n">
-        <f aca="false">MEDIAN(D26:I26)</f>
-        <v>2.09214036220619</v>
-      </c>
-      <c r="E34" s="53" t="n">
-        <f aca="false">QUARTILE(D26:I26,3)</f>
-        <v>2.14147317312342</v>
-      </c>
-      <c r="F34" s="53" t="n">
-        <f aca="false">MEDIAN(D26,E26)</f>
-        <v>2.75652042884463</v>
       </c>
       <c r="G34" s="53" t="n">
         <f aca="false">C26</f>
@@ -16896,32 +17043,39 @@
       </c>
       <c r="H34" s="21" t="n">
         <f aca="false">G34/D34-1</f>
-        <v>0.918673122903492</v>
+        <v>1.18139075968092</v>
+      </c>
+      <c r="I34" s="53" t="n">
+        <f aca="false">D26</f>
+        <v>3.92483787518104</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="16" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B36" s="17" t="s">
+        <v>463</v>
+      </c>
+      <c r="C36" s="17" t="s">
+        <v>455</v>
+      </c>
+      <c r="D36" s="17" t="s">
+        <v>456</v>
+      </c>
+      <c r="E36" s="17" t="s">
+        <v>457</v>
+      </c>
+      <c r="F36" s="17" t="s">
+        <v>458</v>
+      </c>
+      <c r="G36" s="17" t="s">
         <v>461</v>
-      </c>
-      <c r="C36" s="17" t="s">
-        <v>454</v>
-      </c>
-      <c r="D36" s="17" t="s">
-        <v>455</v>
-      </c>
-      <c r="E36" s="17" t="s">
-        <v>456</v>
-      </c>
-      <c r="F36" s="17" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B37" s="23" t="n">
         <f aca="false">C20</f>
@@ -16929,24 +17083,28 @@
       </c>
       <c r="C37" s="56" t="n">
         <f aca="false">(C31*$B37+(C10-C8-C9))/C7</f>
-        <v>208.422465418063</v>
+        <v>216.34231151994</v>
       </c>
       <c r="D37" s="60" t="n">
         <f aca="false">(D31*$B37+(C10-C8-C9))/C7</f>
-        <v>240.101849825571</v>
+        <v>242.819693575233</v>
       </c>
       <c r="E37" s="56" t="n">
         <f aca="false">(E31*$B37+(C10-C8-C9))/C7</f>
-        <v>359.34629792755</v>
+        <v>330.894107776887</v>
       </c>
       <c r="F37" s="56" t="n">
         <f aca="false">(F31*$B37+(C10-C8-C9))/C7</f>
-        <v>452.488830752367</v>
+        <v>359.34629792755</v>
+      </c>
+      <c r="G37" s="56" t="n">
+        <f aca="false">(I31*$B37+(C10-C8-C9))/C7</f>
+        <v>545.631363577184</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B38" s="23" t="n">
         <f aca="false">C11</f>
@@ -16954,24 +17112,28 @@
       </c>
       <c r="C38" s="56" t="n">
         <f aca="false">(C30*$B38+(C10-C8-C9))/C7</f>
-        <v>330.409661486618</v>
+        <v>322.494784853975</v>
       </c>
       <c r="D38" s="60" t="n">
         <f aca="false">(D30*$B38+(C10-C8-C9))/C7</f>
-        <v>384.42207834136</v>
+        <v>362.344418777918</v>
       </c>
       <c r="E38" s="56" t="n">
         <f aca="false">(E30*$B38+(C10-C8-C9))/C7</f>
-        <v>423.009756092804</v>
+        <v>417.506416696804</v>
       </c>
       <c r="F38" s="56" t="n">
         <f aca="false">(F30*$B38+(C10-C8-C9))/C7</f>
-        <v>570.224981344897</v>
+        <v>406.499737904802</v>
+      </c>
+      <c r="G38" s="56" t="n">
+        <f aca="false">(I30*$B38+(C10-C8-C9))/C7</f>
+        <v>733.950224784991</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B39" s="23" t="n">
         <f aca="false">C14</f>
@@ -16979,24 +17141,28 @@
       </c>
       <c r="C39" s="56" t="n">
         <f aca="false">(C32*$B39)/C7</f>
-        <v>251.54102063944</v>
+        <v>258.756788605664</v>
       </c>
       <c r="D39" s="60" t="n">
         <f aca="false">(D32*$B39)/C7</f>
-        <v>280.404092504339</v>
+        <v>313.312330776693</v>
       </c>
       <c r="E39" s="56" t="n">
         <f aca="false">(E32*$B39)/C7</f>
-        <v>408.151966254981</v>
+        <v>392.669116953498</v>
       </c>
       <c r="F39" s="56" t="n">
         <f aca="false">(F32*$B39)/C7</f>
-        <v>547.951826169626</v>
+        <v>408.151966254981</v>
+      </c>
+      <c r="G39" s="56" t="n">
+        <f aca="false">(I32*$B39)/C7</f>
+        <v>687.751686084271</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B40" s="23" t="n">
         <f aca="false">C11</f>
@@ -17004,19 +17170,23 @@
       </c>
       <c r="C40" s="56" t="n">
         <f aca="false">(C33*$B40)/C7</f>
-        <v>245.190303350968</v>
+        <v>263.536006047378</v>
       </c>
       <c r="D40" s="60" t="n">
         <f aca="false">(D33*$B40)/C7</f>
-        <v>324.657184446484</v>
+        <v>326.689203347894</v>
       </c>
       <c r="E40" s="56" t="n">
         <f aca="false">(E33*$B40)/C7</f>
-        <v>370.60900037964</v>
+        <v>363.434986070683</v>
       </c>
       <c r="F40" s="56" t="n">
         <f aca="false">(F33*$B40)/C7</f>
-        <v>531.918506489312</v>
+        <v>377.783014688596</v>
+      </c>
+      <c r="G40" s="56" t="n">
+        <f aca="false">(I33*$B40)/C7</f>
+        <v>686.053998290028</v>
       </c>
     </row>
   </sheetData>

</xml_diff>